<commit_message>
Update Excel add-in workbook
</commit_message>
<xml_diff>
--- a/Excel add-in 8b5f6c3e-83eb-4b93-a97c-0e386bed12c2.xlsx
+++ b/Excel add-in 8b5f6c3e-83eb-4b93-a97c-0e386bed12c2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\Github-Repo\Other Repo\excel-rtd-websocket-addin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{290AB8CD-F0A4-4A8E-B920-215B2520F926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01455D7E-8931-4A79-80C8-E4BDE78DC67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="12">
   <si>
     <t>ACC.NS</t>
   </si>
@@ -38,6 +38,24 @@
   </si>
   <si>
     <t xml:space="preserve">INFY.NS	</t>
+  </si>
+  <si>
+    <t>Symbol</t>
+  </si>
+  <si>
+    <t>LAST</t>
+  </si>
+  <si>
+    <t>OPEN</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>RELIANCE.NS</t>
   </si>
 </sst>
 </file>
@@ -887,7 +905,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="" visibility="1" width="350" row="4">
+  <wetp:taskpane dockstate="" visibility="1" width="542" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -901,6 +919,9 @@
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
   <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions val="1"/>
+    </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
         <we:customFunctionIds>_xldudf_COG_ADD</we:customFunctionIds>
@@ -923,7 +944,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="N14:R16"/>
+  <dimension ref="D14:R24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="15" max="15" width="9" bestFit="1" customWidth="1"/>
@@ -931,7 +952,7 @@
     <col min="18" max="18" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="14" spans="14:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="4:18" x14ac:dyDescent="0.25">
       <c r="O14" t="s">
         <v>1</v>
       </c>
@@ -945,17 +966,32 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="14:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" t="s">
+        <v>8</v>
+      </c>
+      <c r="G15" t="s">
+        <v>9</v>
+      </c>
+      <c r="H15" t="s">
+        <v>10</v>
+      </c>
       <c r="N15" t="s">
         <v>0</v>
       </c>
       <c r="O15" s="1" t="str">
         <f ca="1">_xldudf_COG_GETLIVEDATA(N15,O14)</f>
-        <v>1619.01</v>
-      </c>
-      <c r="P15" s="1" t="e">
+        <v>1633.75</v>
+      </c>
+      <c r="P15" s="1" t="str">
         <f t="shared" ref="P15:R15" ca="1" si="0">_xldudf_COG_GETLIVEDATA(O15,P14)</f>
-        <v>#N/A</v>
+        <v>1689</v>
       </c>
       <c r="Q15" s="1" t="e">
         <f t="shared" ca="1" si="0"/>
@@ -966,17 +1002,36 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="16" spans="14:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="4:18" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("ACC.NS","LAST")</f>
+        <v>1633.75</v>
+      </c>
+      <c r="F16" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("ACC.NS","OPEN")</f>
+        <v>1626</v>
+      </c>
+      <c r="G16" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("ACC.NS","HIGH")</f>
+        <v>1633.75</v>
+      </c>
+      <c r="H16" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("ACC.NS","LOW")</f>
+        <v>1620.43</v>
+      </c>
       <c r="N16" t="s">
         <v>5</v>
       </c>
       <c r="O16" t="str">
         <f ca="1">_xldudf_COG_GETLIVEDATA(N16,O14)</f>
-        <v>1082.01</v>
-      </c>
-      <c r="P16" t="e">
+        <v>1074.88</v>
+      </c>
+      <c r="P16" t="str">
         <f t="shared" ref="P16:R16" ca="1" si="1">_xldudf_COG_GETLIVEDATA(O16,P14)</f>
-        <v>#N/A</v>
+        <v>1692</v>
       </c>
       <c r="Q16" t="e">
         <f t="shared" ca="1" si="1"/>
@@ -985,6 +1040,65 @@
       <c r="R16" t="e">
         <f t="shared" ca="1" si="1"/>
         <v>#N/A</v>
+      </c>
+    </row>
+    <row r="22" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G22" t="s">
+        <v>6</v>
+      </c>
+      <c r="H22" t="s">
+        <v>7</v>
+      </c>
+      <c r="I22" t="s">
+        <v>8</v>
+      </c>
+      <c r="J22" t="s">
+        <v>9</v>
+      </c>
+      <c r="K22" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G23" t="s">
+        <v>0</v>
+      </c>
+      <c r="H23" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("ACC.NS","LAST")</f>
+        <v>1633.75</v>
+      </c>
+      <c r="I23" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("ACC.NS","OPEN")</f>
+        <v>1626</v>
+      </c>
+      <c r="J23" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("ACC.NS","HIGH")</f>
+        <v>1633.75</v>
+      </c>
+      <c r="K23" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("ACC.NS","LOW")</f>
+        <v>1620.43</v>
+      </c>
+    </row>
+    <row r="24" spans="7:11" x14ac:dyDescent="0.25">
+      <c r="G24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("RELIANCE.NS","LAST")</f>
+        <v>1370.58</v>
+      </c>
+      <c r="I24" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("RELIANCE.NS","OPEN")</f>
+        <v>1366</v>
+      </c>
+      <c r="J24" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("RELIANCE.NS","HIGH")</f>
+        <v>1370.58</v>
+      </c>
+      <c r="K24" t="str">
+        <f ca="1">_xldudf_COG_GETLIVEDATA("RELIANCE.NS","LOW")</f>
+        <v>1363.13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>